<commit_message>
A2D Serial Interface working: Reading Data, Reading/Writing Registers; Changes in VHDL and Vitis Project
</commit_message>
<xml_diff>
--- a/IP-Core/Resolver/Registers.xlsx
+++ b/IP-Core/Resolver/Registers.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24701"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga63zix\uz\encoder\IP-Core\Resolver\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixKaiser\Documents\2_EAL_Praktikum_HW\IP-Core\Resolver\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F3E15F-1778-4DA8-9BD3-E904B6AA9511}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11596" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Registers" sheetId="1" r:id="rId1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="83">
   <si>
     <t>RESCON: Resolver Control Register</t>
   </si>
@@ -276,12 +277,18 @@
   </si>
   <si>
     <t>set reset bit</t>
+  </si>
+  <si>
+    <t>Address 3</t>
+  </si>
+  <si>
+    <t>RESRDA: Resolver Register Data Register</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -373,13 +380,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -390,6 +391,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -670,49 +677,49 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:I33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A2:I44"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A2" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+    <row r="3" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A4" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -740,19 +747,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A5" s="9"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A6" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -780,19 +787,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A7" s="9"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A8" s="9" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -820,19 +827,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A9" s="9"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A10" s="9" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -860,8 +867,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A11" s="9"/>
       <c r="B11" s="1" t="s">
         <v>78</v>
       </c>
@@ -887,45 +894,45 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A13" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+    <row r="14" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A14" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="G14" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H14" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="I14" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A15" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -953,19 +960,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="3"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A16" s="9"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A17" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -993,19 +1000,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="3"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A18" s="9"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A19" s="9" t="s">
         <v>4</v>
       </c>
       <c r="B19" s="2" t="s">
@@ -1033,8 +1040,8 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="3"/>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A20" s="9"/>
       <c r="B20" s="1" t="s">
         <v>22</v>
       </c>
@@ -1060,8 +1067,8 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A21" s="9" t="s">
         <v>5</v>
       </c>
       <c r="B21" s="2" t="s">
@@ -1089,8 +1096,8 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="3"/>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A22" s="9"/>
       <c r="B22" s="1" t="s">
         <v>30</v>
       </c>
@@ -1116,45 +1123,45 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A24" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="9" t="s">
+    <row r="25" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A25" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E25" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F25" s="10" t="s">
+      <c r="F25" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G25" s="10" t="s">
+      <c r="G25" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H25" s="10" t="s">
+      <c r="H25" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="I25" s="10" t="s">
+      <c r="I25" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A26" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B26" s="2" t="s">
@@ -1182,19 +1189,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="3"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A27" s="9"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A28" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B28" s="2" t="s">
@@ -1222,19 +1229,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="3"/>
-      <c r="B29" s="7"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="7"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A29" s="9"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A30" s="9" t="s">
         <v>4</v>
       </c>
       <c r="B30" s="2" t="s">
@@ -1262,19 +1269,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="3"/>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A31" s="9"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A32" s="9" t="s">
         <v>5</v>
       </c>
       <c r="B32" s="2" t="s">
@@ -1302,8 +1309,8 @@
         <v>39</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="3"/>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A33" s="9"/>
       <c r="B33" s="1" t="s">
         <v>40</v>
       </c>
@@ -1329,8 +1336,225 @@
         <v>40</v>
       </c>
     </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A35" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A36" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H36" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I36" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A37" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A38" s="9"/>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A39" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A40" s="9"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+      <c r="I40" s="5"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A41" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A42" s="9"/>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5"/>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A43" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A44" s="9"/>
+      <c r="B44" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="16">
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A43:A44"/>
     <mergeCell ref="A32:A33"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="A6:A7"/>
@@ -1350,249 +1574,249 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.28515625" customWidth="1"/>
+    <col min="3" max="3" width="26.265625" customWidth="1"/>
     <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.59765625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.59765625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A1" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="5"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="B1" s="10"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A2" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A3" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A4" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A8" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5" t="s">
+      <c r="B8" s="10"/>
+      <c r="C8" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="5"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="D8" s="10"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A9" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A10" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A11" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A12" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A13" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="4" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A16" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A17" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5" t="s">
+      <c r="B17" s="10"/>
+      <c r="C17" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D17" s="5"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="D17" s="10"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A18" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A19" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="4" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A20" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A21" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="4" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A22" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A23" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="4" t="s">
         <v>52</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C17:D17"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C8:D8"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="C17:D17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>